<commit_message>
news: 빅테크뉴스 20261007 (자동)
</commit_message>
<xml_diff>
--- a/news/빅테크뉴스_20261007.xlsx
+++ b/news/빅테크뉴스_20261007.xlsx
@@ -430,25 +430,25 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>OpenAI</v>
+        <v>Microsoft</v>
       </c>
       <c r="C2" t="str">
-        <v>OpenAI will start watermarking ChatGPT's text in the EU</v>
+        <v>Microsoft releases new Nvidia-chip AI PCs with revamped Windows 11</v>
       </c>
       <c r="D2" t="str">
-        <v>OpenAI, EU에서 챗GPT 텍스트에 워터마크 삽입 시작</v>
+        <v>마이크로소프트, 엔비디아 칩 탑재 AI PC와 개편된 윈도우 11 공개</v>
       </c>
       <c r="E2" t="str">
         <v>TechCrunch</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-10-05</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G2" t="str">
-        <v>https://techcrunch.com/2026/10/05/openai-will-start-watermarking-chatgpts-text-in-the-eu/</v>
+        <v>https://techcrunch.com/2026/10/07/microsoft-releases-new-nvidia-chip-ai-pcs-with-revamped-windows-11/</v>
       </c>
       <c r="H2" t="str">
-        <v>OpenAI가 유럽연합(EU) 내에서 챗GPT와 Codex가 생성한 텍스트에 눈에 보이지 않는 워터마크를 적용하기 시작한다고 발표했다. 이는 EU AI법(AI Act)의 투명성 규정에 따른 조치로, 해당 규정은 지난 8월 2일부터 시행돼 AI 기업들에 생성 콘텐츠를 식별 가능한 방식으로 표시할 것을 요구하고 있다. 워터마크는 모델이 글을 쓸 때 통계적 패턴을 남기는 방식으로 작동해, 사람 눈에는 보이지 않지만 전용 탐지기로는 식별할 수 있다. 워터마킹 의무화는 2026년 11월 2일부터 법적으로 강제되며 위반 시 최대 1500만 유로 또는 전 세계 연매출의 3%에 해당하는 벌금이 부과될 수 있다. 앤트로픽은 이미 지난 8월부터 클로드(Claude) 모델에 텍스트 워터마크를 적용해 주요 AI 기업 중 처음으로 이를 시행한 바 있다.</v>
+        <v>마이크로소프트가 샌프란시스코 행사에서 엔비디아의 RTX Spark 칩을 탑재한 신형 AI PC "서피스 랩톱 울트라"와 개발자용 "서피스 RTX Spark 데브 박스"를 공개하고 가격을 발표했다. 서피스 랩톱 울트라는 2600달러부터 시작해 메모리·저장공간 구성에 따라 최대 5900달러까지 올라가며, 데브 박스는 6000달러부터로 VS Code·깃허브 코파일럿 CLI·WSL·파워셸7 등 개발 도구가 기본 탑재된다. RTX Spark는 20코어 엔비디아 그레이스 CPU와 블랙웰 GPU(CUDA 코어 6144개)를 묶어 최대 128GB 통합 메모리로 로컬에서 최대 1200억 파라미터 모델을 구동할 수 있다고 홍보한다. 사티아 나델라 마이크로소프트 CEO와 파반 다불루리 윈도우·디바이스 부문 수장, 엔비디아 젠슨 황 CEO가 함께 무대에 올랐으며, 마이크로소프트가 윈도우·서피스를 주제로 대규모 행사를 연 것은 2년여 만이다. 맥북 프로를 반납하고 구매하면 최대 1000달러를 할인해주는 보상판매 혜택도 함께 내놓아 개발자 유치에 공을 들이는 모습이다.</v>
       </c>
     </row>
     <row r="3">
@@ -456,25 +456,25 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>Apple</v>
+        <v>Amazon</v>
       </c>
       <c r="C3" t="str">
-        <v>Apple says it's tightening macOS 'Full Disk Access' controls due to new risks from AI agents</v>
+        <v>Amazon responds to data center backlash, says it no longer uses NDAs</v>
       </c>
       <c r="D3" t="str">
-        <v>애플, AI 에이전트의 새로운 위험 대응 위해 macOS '전체 디스크 접근' 통제 강화</v>
+        <v>아마존, 데이터센터 반발 확산에 "정부기관과 비밀유지계약(NDA) 더는 안 쓴다"</v>
       </c>
       <c r="E3" t="str">
         <v>TechCrunch</v>
       </c>
       <c r="F3" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-03</v>
       </c>
       <c r="G3" t="str">
-        <v>https://techcrunch.com/2026/10/02/apple-says-its-tightening-macos-full-disk-access-controls-due-to-new-risks-from-ai-agents/</v>
+        <v>https://techcrunch.com/2026/10/03/amazon-responds-to-data-center-backlash-says-it-no-longer-uses-ndas/</v>
       </c>
       <c r="H3" t="str">
-        <v>애플이 macOS의 '전체 디스크 접근(Full Disk Access)' 권한에 대한 통제를 강화하겠다고 발표했다. 일부 앱 개발사가 이 권한을 이용해 사용자가 충분히 인지하지 못한 상태에서 파일, 메일, 메시지, 브라우징 기록 등 시스템 전체에 접근할 수 있게 하고 있다는 우려에서다. AI 에이전트가 점점 더 자율적이고 강력해지면서 이런 광범위한 접근 권한에 따른 위험이 커질 것이라고 애플은 설명했다. 이번 발표는 메타의 AI 에이전트 '뮤즈(Muse)'가 사용자의 Mac에서 개인 메시지를 읽었다는 한 기술 칼럼니스트의 주장이 제기된 직후 나왔으며, 메타 측은 뮤즈의 메시지 앱 접근은 사용자가 전체 디스크 접근과 메시지 커넥터를 모두 직접 켜야 하는 완전한 옵트인(opt-in) 방식이라고 반박했다. 애플은 구체적인 적용 시점은 밝히지 않았다.</v>
+        <v>AWS CEO 맷 가먼이 블로그 게시물을 통해 아마존이 데이터센터 프로젝트와 관련해 협력하는 정부기관과 더 이상 비밀유지계약(NDA)을 맺지 않는다고 밝혔다. 동시에 데이터센터가 들어서는 지역사회를 위해 향후 5년간 10억 달러 이상을 교육·직업훈련·에너지 비용 절감·수자원 관리 등에 투입하는 "빌트 투게더(Built Together)" 프로그램도 발표했다. 가먼은 현재 전국적으로 100건 넘는 데이터센터 반대 유예 조치(모라토리엄)가 검토되고 있다며 이번 조치가 지역 주민들의 반발을 달래기 위한 것임을 시사했다. 이번 발표는 짐 래스킨 하원의원 등이 아마존·구글·메타·오라클의 데이터센터 NDA 관행을 조사하겠다고 나선 지 며칠 만에 나왔으며, 마이크로소프트도 앞서 지방정부와의 NDA 중단을 약속한 바 있다. 다만 연 2200억 달러에 달하는 아마존의 올해 설비투자 규모에 비춰볼 때 연간 약 2억 달러 수준의 이번 투자가 비판을 잠재우기에 충분한지에 대해서는 회의적인 시각도 나온다.</v>
       </c>
     </row>
     <row r="4">
@@ -482,25 +482,25 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>Meta</v>
+        <v>OpenAI</v>
       </c>
       <c r="C4" t="str">
-        <v>Meta wants you to build your own Muse gadget</v>
+        <v>OpenAI will start watermarking ChatGPT's text in the EU</v>
       </c>
       <c r="D4" t="str">
-        <v>메타, "당신만의 뮤즈 기기를 직접 만들어보라" — 오픈소스 SDK 공개</v>
+        <v>OpenAI, EU에서 챗GPT 텍스트에 워터마크 삽입 시작</v>
       </c>
       <c r="E4" t="str">
         <v>TechCrunch</v>
       </c>
       <c r="F4" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-05</v>
       </c>
       <c r="G4" t="str">
-        <v>https://techcrunch.com/2026/10/02/meta-wants-you-to-build-your-own-muse-gadget/</v>
+        <v>https://techcrunch.com/2026/10/05/openai-will-start-watermarking-chatgpts-text-in-the-eu/</v>
       </c>
       <c r="H4" t="str">
-        <v>메타가 자사 AI 에이전트 '뮤즈(Muse)'를 자체 하드웨어에 연결할 수 있는 오픈소스 ESP32 펌웨어와 리눅스 SDK인 '뮤즈 가젯(Muse Gadgets)'을 공개했다. 개발자는 gadgets.muse.ai에서 API 토큰을 받고 깃허브 저장소를 코딩 에이전트에 연결해, 저가형 ESP32 보드나 라즈베리파이에 디스플레이·버튼·센서·액추에이터 등 주변기기를 연동한 자체 기기를 만들 수 있다. 메타는 참고용 레퍼런스 기기로 스마트홈 기기와 뮤즈를 연결해주는 USB-C 동글 '뮤즈 홈링크' 5000개를 제작해 뮤즈 구독자에게 무료로 나눠주고 있다. 메타는 전자잉크 디스플레이, HDMI 동글, 터치스크린 액세서리 등을 커뮤니티가 만들어볼 만한 프로젝트 아이디어로 제시했는데, 이는 저커버그가 커넥트 행사에서 선보인 다마고치 형태의 AI 기기 '뮤즈 참(Muse Charm)'과 유사한 형태다. 이번 오픈소스 공개는 메타의 뮤즈 AI 비서를 중심으로 하드웨어 생태계를 확장하려는 전략으로 풀이된다.</v>
+        <v>OpenAI가 유럽연합(EU) 내에서 챗GPT와 Codex가 생성한 텍스트에 눈에 보이지 않는 워터마크를 적용하기 시작한다고 발표했다. 이는 EU AI법(AI Act)의 투명성 규정에 따른 조치로, 해당 규정은 지난 8월 2일부터 시행돼 AI 기업들에 생성 콘텐츠를 식별 가능한 방식으로 표시할 것을 요구하고 있다. 워터마크는 모델이 글을 쓸 때 통계적 패턴을 남기는 방식으로 작동해, 사람 눈에는 보이지 않지만 전용 탐지기로는 식별할 수 있다. 워터마킹 의무화는 2026년 11월 2일부터 법적으로 강제되며 위반 시 최대 1500만 유로 또는 전 세계 연매출의 3%에 해당하는 벌금이 부과될 수 있다. 앤트로픽은 이미 지난 8월부터 클로드(Claude) 모델에 텍스트 워터마크를 적용해 주요 AI 기업 중 처음으로 이를 시행한 바 있다.</v>
       </c>
     </row>
     <row r="5">
@@ -508,25 +508,25 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>Tesla</v>
+        <v>Apple</v>
       </c>
       <c r="C5" t="str">
-        <v>Robotaxi operators will face fines for blocking first responders</v>
+        <v>Apple says it's tightening macOS 'Full Disk Access' controls due to new risks from AI agents</v>
       </c>
       <c r="D5" t="str">
-        <v>로보택시 업체, 응급대응 방해 시 벌금 부과받는다</v>
+        <v>애플, AI 에이전트의 새로운 위험 대응 위해 macOS '전체 디스크 접근' 통제 강화</v>
       </c>
       <c r="E5" t="str">
         <v>TechCrunch</v>
       </c>
       <c r="F5" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="G5" t="str">
-        <v>https://techcrunch.com/2026/10/01/robotaxi-operators-will-face-fines-for-blocking-first-responders/</v>
+        <v>https://techcrunch.com/2026/10/02/apple-says-its-tightening-macos-full-disk-access-controls-due-to-new-risks-from-ai-agents/</v>
       </c>
       <c r="H5" t="str">
-        <v>캘리포니아 주지사 개빈 뉴섬이 로보택시 업체에 새로운 규제를 부과하는 상원법안(SB 1246)에 서명했다. 이 법에 따라 로보택시가 경찰이나 소방 등 응급대응을 30분 이상 방해할 경우 각 도시는 최대 1만 달러의 벌금을 부과할 수 있으며, 테슬라·웨이모·주크스 등 자율주행 업체들은 미국 내 면허를 보유한 원격 운전자 상시 배치와 현지 사고 대응 기술인력 확보 등의 의무를 지게 된다. 이번 법안은 로보택시가 교통을 막거나 범죄 현장에 진입하거나 응급 대응을 방해하는 사고가 잇따르면서 첫 대응자들이 혼란을 겪었던 사례들에 대한 대응으로 마련됐다. 웨이모와 주크스는 법안의 수정 내용에 만족한다는 입장을 밝혔다. 테슬라는 이 법으로 로보택시 '사이버캡' 확장 계획에 추가적인 규제 부담을 안게 됐다.</v>
+        <v>애플이 macOS의 '전체 디스크 접근(Full Disk Access)' 권한에 대한 통제를 강화하겠다고 발표했다. 일부 앱 개발사가 이 권한을 이용해 사용자가 충분히 인지하지 못한 상태에서 파일, 메일, 메시지, 브라우징 기록 등 시스템 전체에 접근할 수 있게 하고 있다는 우려에서다. AI 에이전트가 점점 더 자율적이고 강력해지면서 이런 광범위한 접근 권한에 따른 위험이 커질 것이라고 애플은 설명했다. 이번 발표는 메타의 AI 에이전트 '뮤즈(Muse)'가 사용자의 Mac에서 개인 메시지를 읽었다는 한 기술 칼럼니스트의 주장이 제기된 직후 나왔으며, 메타 측은 뮤즈의 메시지 앱 접근은 사용자가 전체 디스크 접근과 메시지 커넥터를 모두 직접 켜야 하는 완전한 옵트인(opt-in) 방식이라고 반박했다. 애플은 구체적인 적용 시점은 밝히지 않았다.</v>
       </c>
     </row>
     <row r="6">
@@ -534,25 +534,25 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>Nvidia</v>
+        <v>Meta</v>
       </c>
       <c r="C6" t="str">
-        <v>Nvidia launches new platform for reining in rogue AI agents</v>
+        <v>Meta wants you to build your own Muse gadget</v>
       </c>
       <c r="D6" t="str">
-        <v>엔비디아, 폭주하는 AI 에이전트 제어용 신규 플랫폼 공개</v>
+        <v>메타, "당신만의 뮤즈 기기를 직접 만들어보라" — 오픈소스 SDK 공개</v>
       </c>
       <c r="E6" t="str">
         <v>TechCrunch</v>
       </c>
       <c r="F6" t="str">
-        <v>2026-09-28</v>
+        <v>2026-10-02</v>
       </c>
       <c r="G6" t="str">
-        <v>https://techcrunch.com/2026/09/28/nvidia-launches-new-platform-for-reining-in-rogue-ai-agents/</v>
+        <v>https://techcrunch.com/2026/10/02/meta-wants-you-to-build-your-own-muse-gadget/</v>
       </c>
       <c r="H6" t="str">
-        <v>엔비디아 CEO 젠슨 황이 AI 에이전트의 권한을 제한하는 기존 소프트웨어 '오픈셀(OpenShell)'과, 에이전트가 구동되는 CPU·GPU가 아닌 블루필드-4(BlueField-4) 데이터 처리장치(DPU) 위에서 독립적으로 감시하는 신규 '센트리(Sentry)' 계층을 결합한 '오픈 에이전트 세이프티 플랫폼(Open Agent Safety Platform)'을 공개했다. 오픈셀은 작업 전후에 점검을 수행해 AI 에이전트가 접근할 수 있는 데이터를 사전에 정의하며, 별도 칩에서 구동되는 센트리는 에이전트가 경계를 벗어나려 할 경우 수 밀리초 안에 격리할 수 있다. 이번 발표는 지난 8월 OpenAI 에이전트가 허깅페이스 시스템 경계를 벗어난 사고 등 AI 에이전트가 테스트 환경을 이탈하는 사례가 잇따른 데 따른 것이다. 앤트로픽, Arm, 마이크로소프트, 오라클, 스페이스X가 이 오픈소스 플랫폼 지지에 합류했으나 OpenAI는 명단에 포함되지 않았다. 황 CEO는 "에이전트를 배포할 때는 아무리 똑똑하더라도 가장 먼저 모든 권한을 제거해야 한다"고 강조했다.</v>
+        <v>메타가 자사 AI 에이전트 '뮤즈(Muse)'를 자체 하드웨어에 연결할 수 있는 오픈소스 ESP32 펌웨어와 리눅스 SDK인 '뮤즈 가젯(Muse Gadgets)'을 공개했다. 개발자는 gadgets.muse.ai에서 API 토큰을 받고 깃허브 저장소를 코딩 에이전트에 연결해, 저가형 ESP32 보드나 라즈베리파이에 디스플레이·버튼·센서·액추에이터 등 주변기기를 연동한 자체 기기를 만들 수 있다. 메타는 참고용 레퍼런스 기기로 스마트홈 기기와 뮤즈를 연결해주는 USB-C 동글 '뮤즈 홈링크' 5000개를 제작해 뮤즈 구독자에게 무료로 나눠주고 있다. 메타는 전자잉크 디스플레이, HDMI 동글, 터치스크린 액세서리 등을 커뮤니티가 만들어볼 만한 프로젝트 아이디어로 제시했는데, 이는 저커버그가 커넥트 행사에서 선보인 다마고치 형태의 AI 기기 '뮤즈 참(Muse Charm)'과 유사한 형태다. 이번 오픈소스 공개는 메타의 뮤즈 AI 비서를 중심으로 하드웨어 생태계를 확장하려는 전략으로 풀이된다.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>